<commit_message>
plot graphs catergory and regon wise in sales and profit
</commit_message>
<xml_diff>
--- a/Analysis_Superstore_Sales/output/superstore_summary.xlsx
+++ b/Analysis_Superstore_Sales/output/superstore_summary.xlsx
@@ -9,6 +9,13 @@
   <sheets>
     <sheet name="Sales by Year" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Monthly Sales" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sales by Category" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Category Sales Year" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Sales by Region" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Region Sales Year" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Profit by Year" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Profit by Category" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Profit by Region" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -709,4 +716,1014 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>sales</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Furniture</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>2406605</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Office Supplies</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>2790258</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2638265</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="B1" t="n">
+        <v>2011</v>
+      </c>
+      <c r="C1" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D1" t="n">
+        <v>2013</v>
+      </c>
+      <c r="E1" t="n">
+        <v>2014</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Furniture</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>170307</v>
+      </c>
+      <c r="C2" t="n">
+        <v>187549</v>
+      </c>
+      <c r="D2" t="n">
+        <v>276168</v>
+      </c>
+      <c r="E2" t="n">
+        <v>299481</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Office Supplies</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>186584</v>
+      </c>
+      <c r="C3" t="n">
+        <v>233625</v>
+      </c>
+      <c r="D3" t="n">
+        <v>296712</v>
+      </c>
+      <c r="E3" t="n">
+        <v>359881</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>194389</v>
+      </c>
+      <c r="C4" t="n">
+        <v>220317</v>
+      </c>
+      <c r="D4" t="n">
+        <v>274355</v>
+      </c>
+      <c r="E4" t="n">
+        <v>375643</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>region</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>sales</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Africa</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>538115</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>50314</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Caribbean</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>251441</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Central</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>1806638</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Central Asia</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>389506</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>575562</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>366492</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>790546</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>North Asia</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>453686</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Oceania</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>625382</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>1031101</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Southeast Asia</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>532172</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>424173</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>region</t>
+        </is>
+      </c>
+      <c r="B1" t="n">
+        <v>2011</v>
+      </c>
+      <c r="C1" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D1" t="n">
+        <v>2013</v>
+      </c>
+      <c r="E1" t="n">
+        <v>2014</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Africa</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>33355</v>
+      </c>
+      <c r="C2" t="n">
+        <v>36724</v>
+      </c>
+      <c r="D2" t="n">
+        <v>57069</v>
+      </c>
+      <c r="E2" t="n">
+        <v>79041</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>4662</v>
+      </c>
+      <c r="C3" t="n">
+        <v>4549</v>
+      </c>
+      <c r="D3" t="n">
+        <v>6681</v>
+      </c>
+      <c r="E3" t="n">
+        <v>5816</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Caribbean</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>14927</v>
+      </c>
+      <c r="C4" t="n">
+        <v>20431</v>
+      </c>
+      <c r="D4" t="n">
+        <v>29307</v>
+      </c>
+      <c r="E4" t="n">
+        <v>38331</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Central</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>139972</v>
+      </c>
+      <c r="C5" t="n">
+        <v>152771</v>
+      </c>
+      <c r="D5" t="n">
+        <v>187205</v>
+      </c>
+      <c r="E5" t="n">
+        <v>226251</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Central Asia</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>26570</v>
+      </c>
+      <c r="C6" t="n">
+        <v>33095</v>
+      </c>
+      <c r="D6" t="n">
+        <v>44236</v>
+      </c>
+      <c r="E6" t="n">
+        <v>51480</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>43840</v>
+      </c>
+      <c r="C7" t="n">
+        <v>48423</v>
+      </c>
+      <c r="D7" t="n">
+        <v>62025</v>
+      </c>
+      <c r="E7" t="n">
+        <v>82985</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>26338</v>
+      </c>
+      <c r="C8" t="n">
+        <v>41314</v>
+      </c>
+      <c r="D8" t="n">
+        <v>42283</v>
+      </c>
+      <c r="E8" t="n">
+        <v>43063</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>42999</v>
+      </c>
+      <c r="C9" t="n">
+        <v>66078</v>
+      </c>
+      <c r="D9" t="n">
+        <v>85191</v>
+      </c>
+      <c r="E9" t="n">
+        <v>112519</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>North Asia</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>40059</v>
+      </c>
+      <c r="C10" t="n">
+        <v>35874</v>
+      </c>
+      <c r="D10" t="n">
+        <v>51362</v>
+      </c>
+      <c r="E10" t="n">
+        <v>50619</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Oceania</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>35765</v>
+      </c>
+      <c r="C11" t="n">
+        <v>51890</v>
+      </c>
+      <c r="D11" t="n">
+        <v>73612</v>
+      </c>
+      <c r="E11" t="n">
+        <v>80513</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>63822</v>
+      </c>
+      <c r="C12" t="n">
+        <v>79961</v>
+      </c>
+      <c r="D12" t="n">
+        <v>107700</v>
+      </c>
+      <c r="E12" t="n">
+        <v>136518</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Southeast Asia</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>41529</v>
+      </c>
+      <c r="C13" t="n">
+        <v>45539</v>
+      </c>
+      <c r="D13" t="n">
+        <v>61807</v>
+      </c>
+      <c r="E13" t="n">
+        <v>71800</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>37442</v>
+      </c>
+      <c r="C14" t="n">
+        <v>24842</v>
+      </c>
+      <c r="D14" t="n">
+        <v>38757</v>
+      </c>
+      <c r="E14" t="n">
+        <v>56069</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>year</t>
+        </is>
+      </c>
+      <c r="B1" t="inlineStr">
+        <is>
+          <t>profit</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="n">
+        <v>2011</v>
+      </c>
+      <c r="B2" t="n">
+        <v>113534.53686</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>2012</v>
+      </c>
+      <c r="B3" t="n">
+        <v>117606.90596</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2013</v>
+      </c>
+      <c r="B4" t="n">
+        <v>169899.98282</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>2014</v>
+      </c>
+      <c r="B5" t="n">
+        <v>176650.86456</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E4"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>category</t>
+        </is>
+      </c>
+      <c r="B1" t="n">
+        <v>2011</v>
+      </c>
+      <c r="C1" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D1" t="n">
+        <v>2013</v>
+      </c>
+      <c r="E1" t="n">
+        <v>2014</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Furniture</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>29691.7777</v>
+      </c>
+      <c r="C2" t="n">
+        <v>24846.0313</v>
+      </c>
+      <c r="D2" t="n">
+        <v>33350.7506</v>
+      </c>
+      <c r="E2" t="n">
+        <v>21494.7966</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Office Supplies</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>33562.4798</v>
+      </c>
+      <c r="C3" t="n">
+        <v>34434.2199</v>
+      </c>
+      <c r="D3" t="n">
+        <v>55551.9571</v>
+      </c>
+      <c r="E3" t="n">
+        <v>76672.1456</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Technology</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>50280.27936</v>
+      </c>
+      <c r="C4" t="n">
+        <v>58326.65476</v>
+      </c>
+      <c r="D4" t="n">
+        <v>80997.27512000001</v>
+      </c>
+      <c r="E4" t="n">
+        <v>78483.92236</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" t="inlineStr">
+        <is>
+          <t>region</t>
+        </is>
+      </c>
+      <c r="B1" t="n">
+        <v>2011</v>
+      </c>
+      <c r="C1" t="n">
+        <v>2012</v>
+      </c>
+      <c r="D1" t="n">
+        <v>2013</v>
+      </c>
+      <c r="E1" t="n">
+        <v>2014</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>Africa</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>3301.287</v>
+      </c>
+      <c r="C2" t="n">
+        <v>6581.613</v>
+      </c>
+      <c r="D2" t="n">
+        <v>9125.370000000001</v>
+      </c>
+      <c r="E2" t="n">
+        <v>11170.941</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Canada</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>740.5799999999999</v>
+      </c>
+      <c r="C3" t="n">
+        <v>2398.23</v>
+      </c>
+      <c r="D3" t="n">
+        <v>1486.41</v>
+      </c>
+      <c r="E3" t="n">
+        <v>1394.16</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Caribbean</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1956.25048</v>
+      </c>
+      <c r="C4" t="n">
+        <v>3272.2836</v>
+      </c>
+      <c r="D4" t="n">
+        <v>3526.88232</v>
+      </c>
+      <c r="E4" t="n">
+        <v>6191.7968</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>Central</t>
+        </is>
+      </c>
+      <c r="B5" t="n">
+        <v>21417.00868</v>
+      </c>
+      <c r="C5" t="n">
+        <v>20845.7417</v>
+      </c>
+      <c r="D5" t="n">
+        <v>38981.39052</v>
+      </c>
+      <c r="E5" t="n">
+        <v>37071.36942</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Central Asia</t>
+        </is>
+      </c>
+      <c r="B6" t="n">
+        <v>8979.975</v>
+      </c>
+      <c r="C6" t="n">
+        <v>13885.146</v>
+      </c>
+      <c r="D6" t="n">
+        <v>14508.687</v>
+      </c>
+      <c r="E6" t="n">
+        <v>18798.858</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>EMEA</t>
+        </is>
+      </c>
+      <c r="B7" t="n">
+        <v>2141.316</v>
+      </c>
+      <c r="C7" t="n">
+        <v>2403.225</v>
+      </c>
+      <c r="D7" t="n">
+        <v>7686.633</v>
+      </c>
+      <c r="E7" t="n">
+        <v>8711.798999999999</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>East</t>
+        </is>
+      </c>
+      <c r="B8" t="n">
+        <v>5632.4972</v>
+      </c>
+      <c r="C8" t="n">
+        <v>13332.9595</v>
+      </c>
+      <c r="D8" t="n">
+        <v>13632.3736</v>
+      </c>
+      <c r="E8" t="n">
+        <v>8876.4213</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>North</t>
+        </is>
+      </c>
+      <c r="B9" t="n">
+        <v>13418.17524</v>
+      </c>
+      <c r="C9" t="n">
+        <v>15906.6362</v>
+      </c>
+      <c r="D9" t="n">
+        <v>16850.95</v>
+      </c>
+      <c r="E9" t="n">
+        <v>18905.4386</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>North Asia</t>
+        </is>
+      </c>
+      <c r="B10" t="n">
+        <v>19662.801</v>
+      </c>
+      <c r="C10" t="n">
+        <v>10404.243</v>
+      </c>
+      <c r="D10" t="n">
+        <v>23037.339</v>
+      </c>
+      <c r="E10" t="n">
+        <v>17597.181</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>Oceania</t>
+        </is>
+      </c>
+      <c r="B11" t="n">
+        <v>14412.213</v>
+      </c>
+      <c r="C11" t="n">
+        <v>12537.405</v>
+      </c>
+      <c r="D11" t="n">
+        <v>12124.339</v>
+      </c>
+      <c r="E11" t="n">
+        <v>9928.031999999999</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>South</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>13342.07066</v>
+      </c>
+      <c r="C12" t="n">
+        <v>8026.75126</v>
+      </c>
+      <c r="D12" t="n">
+        <v>14841.58888</v>
+      </c>
+      <c r="E12" t="n">
+        <v>19055.11784</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Southeast Asia</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>-128.1855000000001</v>
+      </c>
+      <c r="C13" t="n">
+        <v>2915.5962</v>
+      </c>
+      <c r="D13" t="n">
+        <v>2112.3912</v>
+      </c>
+      <c r="E13" t="n">
+        <v>3433.6857</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>West</t>
+        </is>
+      </c>
+      <c r="B14" t="n">
+        <v>8658.5481</v>
+      </c>
+      <c r="C14" t="n">
+        <v>5097.0755</v>
+      </c>
+      <c r="D14" t="n">
+        <v>11985.6283</v>
+      </c>
+      <c r="E14" t="n">
+        <v>15516.0639</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>